<commit_message>
tweaks to template download
</commit_message>
<xml_diff>
--- a/input_template.xlsx
+++ b/input_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://creamlondon-my.sharepoint.com/personal/jamie_creamuk_com/Documents/Documents/GitHub/Cream Bulk UTM Generator/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{18775C05-993D-46CD-AD23-3B8CD8077CA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="8_{18775C05-993D-46CD-AD23-3B8CD8077CA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3FC2FC2F-323B-4907-8799-522CF90F30E9}"/>
   <bookViews>
     <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="11460" xr2:uid="{93A21314-37C0-4433-9B54-5FE9FF03C44D}"/>
   </bookViews>
@@ -36,14 +36,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="24">
   <si>
     <t>Base_URL</t>
   </si>
   <si>
-    <t>https://www.creamuk.com/</t>
-  </si>
-  <si>
     <t>campaign_ID</t>
   </si>
   <si>
@@ -62,56 +59,62 @@
     <t>campaign_content</t>
   </si>
   <si>
-    <t>ch4</t>
-  </si>
-  <si>
-    <t>vod</t>
-  </si>
-  <si>
-    <t>30s</t>
-  </si>
-  <si>
-    <t>abc1_female_45+</t>
-  </si>
-  <si>
-    <t>meta</t>
-  </si>
-  <si>
-    <t>paid-social</t>
-  </si>
-  <si>
-    <t>brand_q1_2026</t>
-  </si>
-  <si>
-    <t>carousel</t>
-  </si>
-  <si>
-    <t>lal_website_traffic_5pc</t>
-  </si>
-  <si>
-    <t>sheerluxe</t>
-  </si>
-  <si>
-    <t>article</t>
-  </si>
-  <si>
-    <t>display</t>
-  </si>
-  <si>
-    <t>300x600</t>
-  </si>
-  <si>
-    <t>hpto</t>
-  </si>
-  <si>
-    <t>300x250</t>
+    <t>https://www.thewhitecompany.com/uk/Primrose-Hill-Eau-de-Toilette--30ml/p/A18070?swatch=No%20Colour</t>
+  </si>
+  <si>
+    <t>https://www.thewhitecompany.com/uk/Primrose-Hill-Hydrating-Hand-and-Body-Wash/p/A18068?swatch=No%20Colour</t>
+  </si>
+  <si>
+    <t>https://www.thewhitecompany.com/uk/Primrose-Hill-Hydrating-Hand-and-Body-Lotion/p/A18069?swatch=No%20Colour</t>
+  </si>
+  <si>
+    <t>https://www.thewhitecompany.com/uk/Primrose-Hill-Luxury-Fragrance-Oil/p/A18024?swatch=No%20Colour</t>
+  </si>
+  <si>
+    <t>https://www.thewhitecompany.com/uk/Primrose-Hill-Luxury-Home-Spray/p/A17758?swatch=No%20Colour</t>
+  </si>
+  <si>
+    <t>https://www.thewhitecompany.com/uk/Primrose-Hill-Luxury-2-Wick-Candle/p/A18507?swatch=No%20Colour</t>
+  </si>
+  <si>
+    <t>https://www.thewhitecompany.com/uk/collection/Primrose-Hill-Edit-Collection/p/primrose-hill-edit-collection</t>
+  </si>
+  <si>
+    <t>CreamSpring26</t>
+  </si>
+  <si>
+    <t>Vogue</t>
+  </si>
+  <si>
+    <t>Article</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EaudeToilette </t>
+  </si>
+  <si>
+    <t>Hand&amp;BodyWash</t>
+  </si>
+  <si>
+    <t>Hand&amp;BodyLotion</t>
+  </si>
+  <si>
+    <t>FragranceOil</t>
+  </si>
+  <si>
+    <t>HomeSpray</t>
+  </si>
+  <si>
+    <t>2WickCandle</t>
+  </si>
+  <si>
+    <t>CTA</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -127,8 +130,22 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -141,8 +158,20 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEBF1DE"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -150,15 +179,42 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -491,7 +547,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CCE51D7E-1CE9-4D90-A24C-EAD1B682E9E0}">
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <cols>
     <col min="1" max="7" width="21.36328125" customWidth="1"/>
@@ -502,134 +558,153 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.75">
-      <c r="A2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2">
-        <v>123</v>
-      </c>
-      <c r="C2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" t="s">
-        <v>9</v>
-      </c>
-      <c r="E2" t="s">
+      <c r="A2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E2" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="F2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G2" t="s">
-        <v>11</v>
+      <c r="G2" s="6" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.75">
-      <c r="A3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3">
-        <v>123</v>
-      </c>
-      <c r="C3" t="s">
-        <v>12</v>
-      </c>
-      <c r="D3" t="s">
-        <v>13</v>
-      </c>
-      <c r="E3" t="s">
+      <c r="A3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E3" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="F3" t="s">
-        <v>15</v>
-      </c>
-      <c r="G3" t="s">
-        <v>16</v>
+      <c r="G3" s="6" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.75">
-      <c r="A4" t="s">
-        <v>1</v>
-      </c>
-      <c r="B4">
-        <v>123</v>
-      </c>
-      <c r="C4" t="s">
-        <v>17</v>
-      </c>
-      <c r="D4" t="s">
-        <v>18</v>
-      </c>
-      <c r="E4" t="s">
+      <c r="A4" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4" s="4" t="s">
         <v>14</v>
+      </c>
+      <c r="G4" s="6" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.75">
-      <c r="A5" t="s">
-        <v>1</v>
-      </c>
-      <c r="B5">
-        <v>123</v>
-      </c>
-      <c r="C5" t="s">
-        <v>17</v>
-      </c>
-      <c r="D5" t="s">
-        <v>19</v>
-      </c>
-      <c r="E5" t="s">
+      <c r="A5" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E5" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="F5" t="s">
-        <v>21</v>
-      </c>
-      <c r="G5" t="s">
+      <c r="G5" s="6" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.75">
-      <c r="A6" t="s">
-        <v>1</v>
-      </c>
-      <c r="B6">
-        <v>123</v>
-      </c>
-      <c r="C6" t="s">
-        <v>17</v>
-      </c>
-      <c r="D6" t="s">
-        <v>19</v>
-      </c>
-      <c r="E6" t="s">
+      <c r="A6" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E6" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="F6" t="s">
+      <c r="G6" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="G6" t="s">
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.75">
+      <c r="A7" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G7" s="6" t="s">
         <v>22</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.75">
+      <c r="A8" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G8" s="8" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1" xr:uid="{863649B2-3048-4583-90A8-B0042AEACA58}"/>
+    <hyperlink ref="A3" r:id="rId2" xr:uid="{611E32E8-F7F5-44FE-AB89-C95B89DFE8F3}"/>
+    <hyperlink ref="A4" r:id="rId3" xr:uid="{AF9082F6-47EF-49B4-9F7A-61849E20596F}"/>
+    <hyperlink ref="A5" r:id="rId4" xr:uid="{8EF8DA2E-61A9-4109-9A0A-A04AA9A52966}"/>
+    <hyperlink ref="A6" r:id="rId5" xr:uid="{2D018876-4DCB-434A-B2C9-BB1879606F67}"/>
+    <hyperlink ref="A7" r:id="rId6" xr:uid="{FFDE05D9-6DBA-4DB5-97E9-D96C384F2515}"/>
+    <hyperlink ref="A8" r:id="rId7" xr:uid="{7BB78804-295C-4C35-8802-91537FBDA814}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>